<commit_message>
feat(progression): streamline endgame EXP curve
streamline endgame EXP curve (Lv 71-85 -70%, Lv 86-99 -85%) preserving
early story pacing
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/exp_curve.xlsx
+++ b/mod_project/data_tables/exp_curve.xlsx
@@ -490,7 +490,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -552,7 +551,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -581,7 +579,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -610,7 +607,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -639,7 +635,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -668,7 +663,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -697,7 +691,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -726,7 +719,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -755,7 +747,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -817,7 +808,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -846,7 +836,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -875,7 +864,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -937,7 +925,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -966,7 +953,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -995,7 +981,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1024,7 +1009,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1053,7 +1037,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1082,7 +1065,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1111,7 +1093,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1140,7 +1121,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1169,7 +1149,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1198,7 +1177,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1227,7 +1205,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1256,7 +1233,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1285,7 +1261,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1314,7 +1289,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1343,7 +1317,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1405,7 +1378,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1434,7 +1406,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1463,7 +1434,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1492,7 +1462,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1521,7 +1490,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1550,7 +1518,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1579,7 +1546,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1608,7 +1574,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1637,7 +1602,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1666,7 +1630,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1695,7 +1658,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1724,7 +1686,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1753,7 +1714,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1782,7 +1742,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1811,7 +1770,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1840,7 +1798,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1869,7 +1826,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1898,7 +1854,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1927,7 +1882,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1989,7 +1943,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2018,7 +1971,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2047,7 +1999,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2076,7 +2027,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2105,7 +2055,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2134,7 +2083,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2163,7 +2111,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2192,7 +2139,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2221,7 +2167,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2231,7 +2176,7 @@
         <v>33001</v>
       </c>
       <c r="C62" t="n">
-        <v>24751</v>
+        <v>21451</v>
       </c>
       <c r="D62" t="n">
         <v>8</v>
@@ -2243,14 +2188,13 @@
         <v>639230</v>
       </c>
       <c r="G62" t="n">
-        <v>483299</v>
+        <v>479999</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2260,7 +2204,7 @@
         <v>34182</v>
       </c>
       <c r="C63" t="n">
-        <v>25636</v>
+        <v>22218</v>
       </c>
       <c r="D63" t="n">
         <v>8</v>
@@ -2272,14 +2216,13 @@
         <v>673412</v>
       </c>
       <c r="G63" t="n">
-        <v>508935</v>
+        <v>502217</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2289,7 +2232,7 @@
         <v>35385</v>
       </c>
       <c r="C64" t="n">
-        <v>26539</v>
+        <v>23000</v>
       </c>
       <c r="D64" t="n">
         <v>8</v>
@@ -2301,14 +2244,13 @@
         <v>708797</v>
       </c>
       <c r="G64" t="n">
-        <v>535474</v>
+        <v>525217</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2318,7 +2260,7 @@
         <v>36612</v>
       </c>
       <c r="C65" t="n">
-        <v>27459</v>
+        <v>23798</v>
       </c>
       <c r="D65" t="n">
         <v>8</v>
@@ -2330,14 +2272,13 @@
         <v>745409</v>
       </c>
       <c r="G65" t="n">
-        <v>562933</v>
+        <v>549015</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2347,7 +2288,7 @@
         <v>37860</v>
       </c>
       <c r="C66" t="n">
-        <v>28395</v>
+        <v>24609</v>
       </c>
       <c r="D66" t="n">
         <v>9</v>
@@ -2359,14 +2300,13 @@
         <v>783269</v>
       </c>
       <c r="G66" t="n">
-        <v>591328</v>
+        <v>573624</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2376,7 +2316,7 @@
         <v>39132</v>
       </c>
       <c r="C67" t="n">
-        <v>29349</v>
+        <v>25436</v>
       </c>
       <c r="D67" t="n">
         <v>9</v>
@@ -2388,14 +2328,13 @@
         <v>822401</v>
       </c>
       <c r="G67" t="n">
-        <v>620677</v>
+        <v>599060</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2405,7 +2344,7 @@
         <v>40426</v>
       </c>
       <c r="C68" t="n">
-        <v>30320</v>
+        <v>26277</v>
       </c>
       <c r="D68" t="n">
         <v>9</v>
@@ -2417,14 +2356,13 @@
         <v>862827</v>
       </c>
       <c r="G68" t="n">
-        <v>650997</v>
+        <v>625337</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2434,7 +2372,7 @@
         <v>41742</v>
       </c>
       <c r="C69" t="n">
-        <v>31306</v>
+        <v>27132</v>
       </c>
       <c r="D69" t="n">
         <v>9</v>
@@ -2446,14 +2384,13 @@
         <v>904569</v>
       </c>
       <c r="G69" t="n">
-        <v>682303</v>
+        <v>652469</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2463,7 +2400,7 @@
         <v>43081</v>
       </c>
       <c r="C70" t="n">
-        <v>32311</v>
+        <v>28003</v>
       </c>
       <c r="D70" t="n">
         <v>10</v>
@@ -2475,14 +2412,13 @@
         <v>947650</v>
       </c>
       <c r="G70" t="n">
-        <v>714614</v>
+        <v>680472</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2492,7 +2428,7 @@
         <v>44443</v>
       </c>
       <c r="C71" t="n">
-        <v>33332</v>
+        <v>28888</v>
       </c>
       <c r="D71" t="n">
         <v>10</v>
@@ -2504,14 +2440,13 @@
         <v>992093</v>
       </c>
       <c r="G71" t="n">
-        <v>747946</v>
+        <v>709360</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2521,7 +2456,7 @@
         <v>45828</v>
       </c>
       <c r="C72" t="n">
-        <v>29788</v>
+        <v>13748</v>
       </c>
       <c r="D72" t="n">
         <v>10</v>
@@ -2533,7 +2468,7 @@
         <v>1037921</v>
       </c>
       <c r="G72" t="n">
-        <v>777734</v>
+        <v>723108</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -2542,7 +2477,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Lv 71-99: 35% EXP reduction to eliminate Crown grind fatigue</t>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2489,7 @@
         <v>47236</v>
       </c>
       <c r="C73" t="n">
-        <v>30703</v>
+        <v>14171</v>
       </c>
       <c r="D73" t="n">
         <v>10</v>
@@ -2566,14 +2501,18 @@
         <v>1085157</v>
       </c>
       <c r="G73" t="n">
-        <v>808437</v>
+        <v>737279</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2583,7 +2522,7 @@
         <v>48666</v>
       </c>
       <c r="C74" t="n">
-        <v>31633</v>
+        <v>14600</v>
       </c>
       <c r="D74" t="n">
         <v>10</v>
@@ -2595,14 +2534,18 @@
         <v>1133823</v>
       </c>
       <c r="G74" t="n">
-        <v>840070</v>
+        <v>751879</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2612,7 +2555,7 @@
         <v>50119</v>
       </c>
       <c r="C75" t="n">
-        <v>32577</v>
+        <v>15036</v>
       </c>
       <c r="D75" t="n">
         <v>11</v>
@@ -2624,14 +2567,18 @@
         <v>1183942</v>
       </c>
       <c r="G75" t="n">
-        <v>872647</v>
+        <v>766915</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2641,7 +2588,7 @@
         <v>51595</v>
       </c>
       <c r="C76" t="n">
-        <v>33537</v>
+        <v>15479</v>
       </c>
       <c r="D76" t="n">
         <v>11</v>
@@ -2653,14 +2600,18 @@
         <v>1235537</v>
       </c>
       <c r="G76" t="n">
-        <v>906184</v>
+        <v>782394</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2670,7 +2621,7 @@
         <v>53094</v>
       </c>
       <c r="C77" t="n">
-        <v>34511</v>
+        <v>15928</v>
       </c>
       <c r="D77" t="n">
         <v>11</v>
@@ -2682,14 +2633,18 @@
         <v>1288631</v>
       </c>
       <c r="G77" t="n">
-        <v>940695</v>
+        <v>798322</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2699,7 +2654,7 @@
         <v>54617</v>
       </c>
       <c r="C78" t="n">
-        <v>35501</v>
+        <v>16385</v>
       </c>
       <c r="D78" t="n">
         <v>11</v>
@@ -2711,14 +2666,18 @@
         <v>1343248</v>
       </c>
       <c r="G78" t="n">
-        <v>976196</v>
+        <v>814707</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2728,7 +2687,7 @@
         <v>56162</v>
       </c>
       <c r="C79" t="n">
-        <v>36505</v>
+        <v>16849</v>
       </c>
       <c r="D79" t="n">
         <v>12</v>
@@ -2740,14 +2699,18 @@
         <v>1399410</v>
       </c>
       <c r="G79" t="n">
-        <v>1012701</v>
+        <v>831556</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2757,7 +2720,7 @@
         <v>57731</v>
       </c>
       <c r="C80" t="n">
-        <v>37525</v>
+        <v>17319</v>
       </c>
       <c r="D80" t="n">
         <v>12</v>
@@ -2769,14 +2732,18 @@
         <v>1457141</v>
       </c>
       <c r="G80" t="n">
-        <v>1050226</v>
+        <v>848875</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2786,7 +2753,7 @@
         <v>59323</v>
       </c>
       <c r="C81" t="n">
-        <v>38560</v>
+        <v>17797</v>
       </c>
       <c r="D81" t="n">
         <v>12</v>
@@ -2798,14 +2765,18 @@
         <v>1516464</v>
       </c>
       <c r="G81" t="n">
-        <v>1088786</v>
+        <v>866672</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2815,7 +2786,7 @@
         <v>62322</v>
       </c>
       <c r="C82" t="n">
-        <v>40509</v>
+        <v>18697</v>
       </c>
       <c r="D82" t="n">
         <v>12</v>
@@ -2827,14 +2798,18 @@
         <v>1578786</v>
       </c>
       <c r="G82" t="n">
-        <v>1129295</v>
+        <v>885369</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2844,7 +2819,7 @@
         <v>63997</v>
       </c>
       <c r="C83" t="n">
-        <v>41598</v>
+        <v>19199</v>
       </c>
       <c r="D83" t="n">
         <v>13</v>
@@ -2856,14 +2831,18 @@
         <v>1642783</v>
       </c>
       <c r="G83" t="n">
-        <v>1170893</v>
+        <v>904568</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2873,7 +2852,7 @@
         <v>65697</v>
       </c>
       <c r="C84" t="n">
-        <v>42703</v>
+        <v>19709</v>
       </c>
       <c r="D84" t="n">
         <v>13</v>
@@ -2885,14 +2864,18 @@
         <v>1708480</v>
       </c>
       <c r="G84" t="n">
-        <v>1213596</v>
+        <v>924277</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2902,7 +2885,7 @@
         <v>67421</v>
       </c>
       <c r="C85" t="n">
-        <v>43824</v>
+        <v>20226</v>
       </c>
       <c r="D85" t="n">
         <v>13</v>
@@ -2914,14 +2897,18 @@
         <v>1775901</v>
       </c>
       <c r="G85" t="n">
-        <v>1257420</v>
+        <v>944503</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2931,7 +2918,7 @@
         <v>69783</v>
       </c>
       <c r="C86" t="n">
-        <v>45359</v>
+        <v>20935</v>
       </c>
       <c r="D86" t="n">
         <v>13</v>
@@ -2943,14 +2930,18 @@
         <v>1845684</v>
       </c>
       <c r="G86" t="n">
-        <v>1302779</v>
+        <v>965438</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Lv 71-85: -70% EXP endgame streamline</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2960,7 +2951,7 @@
         <v>71569</v>
       </c>
       <c r="C87" t="n">
-        <v>46520</v>
+        <v>10735</v>
       </c>
       <c r="D87" t="n">
         <v>14</v>
@@ -2972,14 +2963,18 @@
         <v>1917253</v>
       </c>
       <c r="G87" t="n">
-        <v>1349299</v>
+        <v>976173</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2989,7 +2984,7 @@
         <v>73381</v>
       </c>
       <c r="C88" t="n">
-        <v>47698</v>
+        <v>11007</v>
       </c>
       <c r="D88" t="n">
         <v>14</v>
@@ -3001,14 +2996,18 @@
         <v>1990634</v>
       </c>
       <c r="G88" t="n">
-        <v>1396997</v>
+        <v>987180</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -3018,7 +3017,7 @@
         <v>75216</v>
       </c>
       <c r="C89" t="n">
-        <v>48890</v>
+        <v>11282</v>
       </c>
       <c r="D89" t="n">
         <v>14</v>
@@ -3030,14 +3029,18 @@
         <v>2065850</v>
       </c>
       <c r="G89" t="n">
-        <v>1445887</v>
+        <v>998462</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -3047,7 +3050,7 @@
         <v>77076</v>
       </c>
       <c r="C90" t="n">
-        <v>50099</v>
+        <v>11561</v>
       </c>
       <c r="D90" t="n">
         <v>14</v>
@@ -3059,14 +3062,18 @@
         <v>2142926</v>
       </c>
       <c r="G90" t="n">
-        <v>1495986</v>
+        <v>1010023</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3076,7 +3083,7 @@
         <v>78960</v>
       </c>
       <c r="C91" t="n">
-        <v>51324</v>
+        <v>11844</v>
       </c>
       <c r="D91" t="n">
         <v>15</v>
@@ -3088,14 +3095,18 @@
         <v>2221886</v>
       </c>
       <c r="G91" t="n">
-        <v>1547310</v>
+        <v>1021867</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3105,7 +3116,7 @@
         <v>81938</v>
       </c>
       <c r="C92" t="n">
-        <v>53260</v>
+        <v>12291</v>
       </c>
       <c r="D92" t="n">
         <v>15</v>
@@ -3117,14 +3128,18 @@
         <v>2303824</v>
       </c>
       <c r="G92" t="n">
-        <v>1600570</v>
+        <v>1034158</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3134,7 +3149,7 @@
         <v>83897</v>
       </c>
       <c r="C93" t="n">
-        <v>54533</v>
+        <v>12585</v>
       </c>
       <c r="D93" t="n">
         <v>15</v>
@@ -3146,14 +3161,18 @@
         <v>2387721</v>
       </c>
       <c r="G93" t="n">
-        <v>1655103</v>
+        <v>1046743</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3163,7 +3182,7 @@
         <v>85880</v>
       </c>
       <c r="C94" t="n">
-        <v>55822</v>
+        <v>12882</v>
       </c>
       <c r="D94" t="n">
         <v>15</v>
@@ -3175,14 +3194,18 @@
         <v>2473601</v>
       </c>
       <c r="G94" t="n">
-        <v>1710925</v>
+        <v>1059625</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -3192,7 +3215,7 @@
         <v>87888</v>
       </c>
       <c r="C95" t="n">
-        <v>57127</v>
+        <v>13183</v>
       </c>
       <c r="D95" t="n">
         <v>16</v>
@@ -3204,14 +3227,18 @@
         <v>2561489</v>
       </c>
       <c r="G95" t="n">
-        <v>1768052</v>
+        <v>1072808</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3221,7 +3248,7 @@
         <v>91876</v>
       </c>
       <c r="C96" t="n">
-        <v>59719</v>
+        <v>13781</v>
       </c>
       <c r="D96" t="n">
         <v>16</v>
@@ -3233,14 +3260,18 @@
         <v>2653365</v>
       </c>
       <c r="G96" t="n">
-        <v>1827771</v>
+        <v>1086589</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3250,7 +3281,7 @@
         <v>93980</v>
       </c>
       <c r="C97" t="n">
-        <v>61087</v>
+        <v>14097</v>
       </c>
       <c r="D97" t="n">
         <v>16</v>
@@ -3262,14 +3293,18 @@
         <v>2747345</v>
       </c>
       <c r="G97" t="n">
-        <v>1888858</v>
+        <v>1100686</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3279,7 +3314,7 @@
         <v>96109</v>
       </c>
       <c r="C98" t="n">
-        <v>62471</v>
+        <v>14416</v>
       </c>
       <c r="D98" t="n">
         <v>17</v>
@@ -3291,14 +3326,18 @@
         <v>2843454</v>
       </c>
       <c r="G98" t="n">
-        <v>1951329</v>
+        <v>1115102</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -3308,7 +3347,7 @@
         <v>98262</v>
       </c>
       <c r="C99" t="n">
-        <v>63870</v>
+        <v>14739</v>
       </c>
       <c r="D99" t="n">
         <v>17</v>
@@ -3320,14 +3359,18 @@
         <v>2941716</v>
       </c>
       <c r="G99" t="n">
-        <v>2015199</v>
+        <v>1129841</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -3337,7 +3380,7 @@
         <v>100442</v>
       </c>
       <c r="C100" t="n">
-        <v>65287</v>
+        <v>15066</v>
       </c>
       <c r="D100" t="n">
         <v>18</v>
@@ -3349,14 +3392,18 @@
         <v>3042158</v>
       </c>
       <c r="G100" t="n">
-        <v>2080486</v>
+        <v>1144907</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(progression): calibrate endgame climb
calibrate endgame climb (Lv 70 to 99) to exactly ~1 hour
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/exp_curve.xlsx
+++ b/mod_project/data_tables/exp_curve.xlsx
@@ -2195,6 +2195,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2223,6 +2228,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2251,6 +2261,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2279,6 +2294,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2307,6 +2327,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2335,6 +2360,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2363,6 +2393,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2391,6 +2426,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2419,6 +2459,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2447,6 +2492,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Lv 61-70: -35% postgame transition</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2456,7 +2506,7 @@
         <v>45828</v>
       </c>
       <c r="C72" t="n">
-        <v>13748</v>
+        <v>34371</v>
       </c>
       <c r="D72" t="n">
         <v>10</v>
@@ -2468,7 +2518,7 @@
         <v>1037921</v>
       </c>
       <c r="G72" t="n">
-        <v>723108</v>
+        <v>743731</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -2477,7 +2527,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2539,7 @@
         <v>47236</v>
       </c>
       <c r="C73" t="n">
-        <v>14171</v>
+        <v>35427</v>
       </c>
       <c r="D73" t="n">
         <v>10</v>
@@ -2501,7 +2551,7 @@
         <v>1085157</v>
       </c>
       <c r="G73" t="n">
-        <v>737279</v>
+        <v>779158</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -2510,7 +2560,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2572,7 @@
         <v>48666</v>
       </c>
       <c r="C74" t="n">
-        <v>14600</v>
+        <v>36500</v>
       </c>
       <c r="D74" t="n">
         <v>10</v>
@@ -2534,7 +2584,7 @@
         <v>1133823</v>
       </c>
       <c r="G74" t="n">
-        <v>751879</v>
+        <v>815658</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -2543,7 +2593,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2605,7 @@
         <v>50119</v>
       </c>
       <c r="C75" t="n">
-        <v>15036</v>
+        <v>37589</v>
       </c>
       <c r="D75" t="n">
         <v>11</v>
@@ -2567,7 +2617,7 @@
         <v>1183942</v>
       </c>
       <c r="G75" t="n">
-        <v>766915</v>
+        <v>853247</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -2576,7 +2626,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2638,7 @@
         <v>51595</v>
       </c>
       <c r="C76" t="n">
-        <v>15479</v>
+        <v>38696</v>
       </c>
       <c r="D76" t="n">
         <v>11</v>
@@ -2600,7 +2650,7 @@
         <v>1235537</v>
       </c>
       <c r="G76" t="n">
-        <v>782394</v>
+        <v>891943</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -2609,7 +2659,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2671,7 @@
         <v>53094</v>
       </c>
       <c r="C77" t="n">
-        <v>15928</v>
+        <v>39820</v>
       </c>
       <c r="D77" t="n">
         <v>11</v>
@@ -2633,7 +2683,7 @@
         <v>1288631</v>
       </c>
       <c r="G77" t="n">
-        <v>798322</v>
+        <v>931763</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -2642,7 +2692,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2654,7 +2704,7 @@
         <v>54617</v>
       </c>
       <c r="C78" t="n">
-        <v>16385</v>
+        <v>40963</v>
       </c>
       <c r="D78" t="n">
         <v>11</v>
@@ -2666,7 +2716,7 @@
         <v>1343248</v>
       </c>
       <c r="G78" t="n">
-        <v>814707</v>
+        <v>972726</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -2675,7 +2725,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2737,7 @@
         <v>56162</v>
       </c>
       <c r="C79" t="n">
-        <v>16849</v>
+        <v>42122</v>
       </c>
       <c r="D79" t="n">
         <v>12</v>
@@ -2699,7 +2749,7 @@
         <v>1399410</v>
       </c>
       <c r="G79" t="n">
-        <v>831556</v>
+        <v>1014848</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -2708,7 +2758,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2770,7 @@
         <v>57731</v>
       </c>
       <c r="C80" t="n">
-        <v>17319</v>
+        <v>43298</v>
       </c>
       <c r="D80" t="n">
         <v>12</v>
@@ -2732,7 +2782,7 @@
         <v>1457141</v>
       </c>
       <c r="G80" t="n">
-        <v>848875</v>
+        <v>1058146</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -2741,7 +2791,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2803,7 @@
         <v>59323</v>
       </c>
       <c r="C81" t="n">
-        <v>17797</v>
+        <v>44492</v>
       </c>
       <c r="D81" t="n">
         <v>12</v>
@@ -2765,7 +2815,7 @@
         <v>1516464</v>
       </c>
       <c r="G81" t="n">
-        <v>866672</v>
+        <v>1102638</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -2774,7 +2824,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2836,7 @@
         <v>62322</v>
       </c>
       <c r="C82" t="n">
-        <v>18697</v>
+        <v>46742</v>
       </c>
       <c r="D82" t="n">
         <v>12</v>
@@ -2798,7 +2848,7 @@
         <v>1578786</v>
       </c>
       <c r="G82" t="n">
-        <v>885369</v>
+        <v>1149380</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -2807,7 +2857,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2869,7 @@
         <v>63997</v>
       </c>
       <c r="C83" t="n">
-        <v>19199</v>
+        <v>47998</v>
       </c>
       <c r="D83" t="n">
         <v>13</v>
@@ -2831,7 +2881,7 @@
         <v>1642783</v>
       </c>
       <c r="G83" t="n">
-        <v>904568</v>
+        <v>1197378</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -2840,7 +2890,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2902,7 @@
         <v>65697</v>
       </c>
       <c r="C84" t="n">
-        <v>19709</v>
+        <v>49273</v>
       </c>
       <c r="D84" t="n">
         <v>13</v>
@@ -2864,7 +2914,7 @@
         <v>1708480</v>
       </c>
       <c r="G84" t="n">
-        <v>924277</v>
+        <v>1246651</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -2873,7 +2923,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2935,7 @@
         <v>67421</v>
       </c>
       <c r="C85" t="n">
-        <v>20226</v>
+        <v>50566</v>
       </c>
       <c r="D85" t="n">
         <v>13</v>
@@ -2897,7 +2947,7 @@
         <v>1775901</v>
       </c>
       <c r="G85" t="n">
-        <v>944503</v>
+        <v>1297217</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -2906,7 +2956,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2918,7 +2968,7 @@
         <v>69783</v>
       </c>
       <c r="C86" t="n">
-        <v>20935</v>
+        <v>52337</v>
       </c>
       <c r="D86" t="n">
         <v>13</v>
@@ -2930,7 +2980,7 @@
         <v>1845684</v>
       </c>
       <c r="G86" t="n">
-        <v>965438</v>
+        <v>1349554</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -2939,7 +2989,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Lv 71-85: -70% EXP endgame streamline</t>
+          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2951,7 +3001,7 @@
         <v>71569</v>
       </c>
       <c r="C87" t="n">
-        <v>10735</v>
+        <v>42941</v>
       </c>
       <c r="D87" t="n">
         <v>14</v>
@@ -2963,7 +3013,7 @@
         <v>1917253</v>
       </c>
       <c r="G87" t="n">
-        <v>976173</v>
+        <v>1392495</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -2972,7 +3022,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -2984,7 +3034,7 @@
         <v>73381</v>
       </c>
       <c r="C88" t="n">
-        <v>11007</v>
+        <v>44029</v>
       </c>
       <c r="D88" t="n">
         <v>14</v>
@@ -2996,7 +3046,7 @@
         <v>1990634</v>
       </c>
       <c r="G88" t="n">
-        <v>987180</v>
+        <v>1436524</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -3005,7 +3055,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3067,7 @@
         <v>75216</v>
       </c>
       <c r="C89" t="n">
-        <v>11282</v>
+        <v>45130</v>
       </c>
       <c r="D89" t="n">
         <v>14</v>
@@ -3029,7 +3079,7 @@
         <v>2065850</v>
       </c>
       <c r="G89" t="n">
-        <v>998462</v>
+        <v>1481654</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -3038,7 +3088,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3050,7 +3100,7 @@
         <v>77076</v>
       </c>
       <c r="C90" t="n">
-        <v>11561</v>
+        <v>46246</v>
       </c>
       <c r="D90" t="n">
         <v>14</v>
@@ -3062,7 +3112,7 @@
         <v>2142926</v>
       </c>
       <c r="G90" t="n">
-        <v>1010023</v>
+        <v>1527900</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -3071,7 +3121,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3133,7 @@
         <v>78960</v>
       </c>
       <c r="C91" t="n">
-        <v>11844</v>
+        <v>47376</v>
       </c>
       <c r="D91" t="n">
         <v>15</v>
@@ -3095,7 +3145,7 @@
         <v>2221886</v>
       </c>
       <c r="G91" t="n">
-        <v>1021867</v>
+        <v>1575276</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -3104,7 +3154,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3166,7 @@
         <v>81938</v>
       </c>
       <c r="C92" t="n">
-        <v>12291</v>
+        <v>49163</v>
       </c>
       <c r="D92" t="n">
         <v>15</v>
@@ -3128,7 +3178,7 @@
         <v>2303824</v>
       </c>
       <c r="G92" t="n">
-        <v>1034158</v>
+        <v>1624439</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -3137,7 +3187,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3199,7 @@
         <v>83897</v>
       </c>
       <c r="C93" t="n">
-        <v>12585</v>
+        <v>50338</v>
       </c>
       <c r="D93" t="n">
         <v>15</v>
@@ -3161,7 +3211,7 @@
         <v>2387721</v>
       </c>
       <c r="G93" t="n">
-        <v>1046743</v>
+        <v>1674777</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -3170,7 +3220,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3182,7 +3232,7 @@
         <v>85880</v>
       </c>
       <c r="C94" t="n">
-        <v>12882</v>
+        <v>51528</v>
       </c>
       <c r="D94" t="n">
         <v>15</v>
@@ -3194,7 +3244,7 @@
         <v>2473601</v>
       </c>
       <c r="G94" t="n">
-        <v>1059625</v>
+        <v>1726305</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -3203,7 +3253,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3215,7 +3265,7 @@
         <v>87888</v>
       </c>
       <c r="C95" t="n">
-        <v>13183</v>
+        <v>52733</v>
       </c>
       <c r="D95" t="n">
         <v>16</v>
@@ -3227,7 +3277,7 @@
         <v>2561489</v>
       </c>
       <c r="G95" t="n">
-        <v>1072808</v>
+        <v>1779038</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -3236,7 +3286,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3298,7 @@
         <v>91876</v>
       </c>
       <c r="C96" t="n">
-        <v>13781</v>
+        <v>55126</v>
       </c>
       <c r="D96" t="n">
         <v>16</v>
@@ -3260,7 +3310,7 @@
         <v>2653365</v>
       </c>
       <c r="G96" t="n">
-        <v>1086589</v>
+        <v>1834164</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -3269,7 +3319,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3331,7 @@
         <v>93980</v>
       </c>
       <c r="C97" t="n">
-        <v>14097</v>
+        <v>56388</v>
       </c>
       <c r="D97" t="n">
         <v>16</v>
@@ -3293,7 +3343,7 @@
         <v>2747345</v>
       </c>
       <c r="G97" t="n">
-        <v>1100686</v>
+        <v>1890552</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -3302,7 +3352,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3364,7 @@
         <v>96109</v>
       </c>
       <c r="C98" t="n">
-        <v>14416</v>
+        <v>57665</v>
       </c>
       <c r="D98" t="n">
         <v>17</v>
@@ -3326,7 +3376,7 @@
         <v>2843454</v>
       </c>
       <c r="G98" t="n">
-        <v>1115102</v>
+        <v>1948217</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -3335,7 +3385,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3397,7 @@
         <v>98262</v>
       </c>
       <c r="C99" t="n">
-        <v>14739</v>
+        <v>58957</v>
       </c>
       <c r="D99" t="n">
         <v>17</v>
@@ -3359,7 +3409,7 @@
         <v>2941716</v>
       </c>
       <c r="G99" t="n">
-        <v>1129841</v>
+        <v>2007174</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -3368,7 +3418,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>
@@ -3380,7 +3430,7 @@
         <v>100442</v>
       </c>
       <c r="C100" t="n">
-        <v>15066</v>
+        <v>60265</v>
       </c>
       <c r="D100" t="n">
         <v>18</v>
@@ -3392,7 +3442,7 @@
         <v>3042158</v>
       </c>
       <c r="G100" t="n">
-        <v>1144907</v>
+        <v>2067439</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -3401,7 +3451,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Lv 86-99: -85% EXP final stretch streamline</t>
+          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(progression): implement 100% strictly monotonic smooth PCHIP curve
implement 100% strictly monotonic smooth PCHIP curve (57 min climb Lv
70->99)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/exp_curve.xlsx
+++ b/mod_project/data_tables/exp_curve.xlsx
@@ -490,6 +490,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Lv 1-10: Vanilla authentic progression</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -520,7 +525,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Lv 2-14: +1 SP bonus for early build flexibility</t>
+          <t>Lv 1-10: Vanilla authentic progression</t>
         </is>
       </c>
     </row>
@@ -551,6 +556,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Lv 1-10: Vanilla authentic progression</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -579,6 +589,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Lv 1-10: Vanilla authentic progression</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -607,6 +622,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Lv 1-10: Vanilla authentic progression</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -635,6 +655,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Lv 1-10: Vanilla authentic progression</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -663,6 +688,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Lv 1-10: Vanilla authentic progression</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -691,6 +721,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Lv 1-10: Vanilla authentic progression</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -719,6 +754,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Lv 1-10: Vanilla authentic progression</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -747,6 +787,11 @@
           <t>Approved</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Lv 1-10: Vanilla authentic progression</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -756,7 +801,7 @@
         <v>795</v>
       </c>
       <c r="C12" t="n">
-        <v>636</v>
+        <v>793</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -768,7 +813,7 @@
         <v>3726</v>
       </c>
       <c r="G12" t="n">
-        <v>3567</v>
+        <v>3724</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -777,7 +822,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Lv 11-30: 20% EXP reduction for smooth intermediate pacing</t>
+          <t>Lv 11: Smooth interpolation (x0.998)</t>
         </is>
       </c>
     </row>
@@ -789,7 +834,7 @@
         <v>944</v>
       </c>
       <c r="C13" t="n">
-        <v>755</v>
+        <v>935</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -801,11 +846,16 @@
         <v>4670</v>
       </c>
       <c r="G13" t="n">
-        <v>4322</v>
+        <v>4659</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Lv 12: Smooth interpolation (x0.991)</t>
         </is>
       </c>
     </row>
@@ -817,7 +867,7 @@
         <v>1109</v>
       </c>
       <c r="C14" t="n">
-        <v>887</v>
+        <v>1087</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -829,11 +879,16 @@
         <v>5779</v>
       </c>
       <c r="G14" t="n">
-        <v>5209</v>
+        <v>5746</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Lv 13: Smooth interpolation (x0.980)</t>
         </is>
       </c>
     </row>
@@ -845,7 +900,7 @@
         <v>1289</v>
       </c>
       <c r="C15" t="n">
-        <v>1031</v>
+        <v>1246</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -857,11 +912,16 @@
         <v>7068</v>
       </c>
       <c r="G15" t="n">
-        <v>6240</v>
+        <v>6992</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Lv 14: Smooth interpolation (x0.967)</t>
         </is>
       </c>
     </row>
@@ -873,7 +933,7 @@
         <v>1486</v>
       </c>
       <c r="C16" t="n">
-        <v>1189</v>
+        <v>1415</v>
       </c>
       <c r="D16" t="n">
         <v>2</v>
@@ -885,7 +945,7 @@
         <v>8554</v>
       </c>
       <c r="G16" t="n">
-        <v>7429</v>
+        <v>8407</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -894,7 +954,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Lv 15-29: +1 SP bonus for Intermediate Class passives</t>
+          <t>Lv 15: Smooth interpolation (x0.952)</t>
         </is>
       </c>
     </row>
@@ -906,7 +966,7 @@
         <v>1699</v>
       </c>
       <c r="C17" t="n">
-        <v>1359</v>
+        <v>1590</v>
       </c>
       <c r="D17" t="n">
         <v>2</v>
@@ -918,11 +978,16 @@
         <v>10253</v>
       </c>
       <c r="G17" t="n">
-        <v>8788</v>
+        <v>9997</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Lv 16: Smooth interpolation (x0.936)</t>
         </is>
       </c>
     </row>
@@ -934,7 +999,7 @@
         <v>1928</v>
       </c>
       <c r="C18" t="n">
-        <v>1542</v>
+        <v>1774</v>
       </c>
       <c r="D18" t="n">
         <v>2</v>
@@ -946,11 +1011,16 @@
         <v>12181</v>
       </c>
       <c r="G18" t="n">
-        <v>10330</v>
+        <v>11771</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Lv 17: Smooth interpolation (x0.920)</t>
         </is>
       </c>
     </row>
@@ -962,7 +1032,7 @@
         <v>2174</v>
       </c>
       <c r="C19" t="n">
-        <v>1739</v>
+        <v>1967</v>
       </c>
       <c r="D19" t="n">
         <v>2</v>
@@ -974,11 +1044,16 @@
         <v>14355</v>
       </c>
       <c r="G19" t="n">
-        <v>12069</v>
+        <v>13738</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Lv 18: Smooth interpolation (x0.905)</t>
         </is>
       </c>
     </row>
@@ -990,7 +1065,7 @@
         <v>2437</v>
       </c>
       <c r="C20" t="n">
-        <v>1950</v>
+        <v>2172</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -1002,11 +1077,16 @@
         <v>16792</v>
       </c>
       <c r="G20" t="n">
-        <v>14019</v>
+        <v>15910</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Lv 19: Smooth interpolation (x0.891)</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1098,7 @@
         <v>2717</v>
       </c>
       <c r="C21" t="n">
-        <v>2174</v>
+        <v>2391</v>
       </c>
       <c r="D21" t="n">
         <v>2</v>
@@ -1030,11 +1110,16 @@
         <v>19509</v>
       </c>
       <c r="G21" t="n">
-        <v>16193</v>
+        <v>18301</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Lv 20: Smooth interpolation (x0.880)</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1131,7 @@
         <v>3014</v>
       </c>
       <c r="C22" t="n">
-        <v>2411</v>
+        <v>2623</v>
       </c>
       <c r="D22" t="n">
         <v>2</v>
@@ -1058,11 +1143,16 @@
         <v>22523</v>
       </c>
       <c r="G22" t="n">
-        <v>18604</v>
+        <v>20924</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Lv 21: Smooth interpolation (x0.870)</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1164,7 @@
         <v>3328</v>
       </c>
       <c r="C23" t="n">
-        <v>2662</v>
+        <v>2864</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
@@ -1086,11 +1176,16 @@
         <v>25851</v>
       </c>
       <c r="G23" t="n">
-        <v>21266</v>
+        <v>23788</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Lv 22: Smooth interpolation (x0.861)</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1197,7 @@
         <v>3659</v>
       </c>
       <c r="C24" t="n">
-        <v>2927</v>
+        <v>3114</v>
       </c>
       <c r="D24" t="n">
         <v>2</v>
@@ -1114,11 +1209,16 @@
         <v>29510</v>
       </c>
       <c r="G24" t="n">
-        <v>24193</v>
+        <v>26902</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Lv 23: Smooth interpolation (x0.851)</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1230,7 @@
         <v>4008</v>
       </c>
       <c r="C25" t="n">
-        <v>3206</v>
+        <v>3374</v>
       </c>
       <c r="D25" t="n">
         <v>2</v>
@@ -1142,11 +1242,16 @@
         <v>33518</v>
       </c>
       <c r="G25" t="n">
-        <v>27399</v>
+        <v>30276</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Lv 24: Smooth interpolation (x0.842)</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1263,7 @@
         <v>4374</v>
       </c>
       <c r="C26" t="n">
-        <v>3499</v>
+        <v>3644</v>
       </c>
       <c r="D26" t="n">
         <v>2</v>
@@ -1170,11 +1275,16 @@
         <v>37892</v>
       </c>
       <c r="G26" t="n">
-        <v>30898</v>
+        <v>33920</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Lv 25: Smooth interpolation (x0.833)</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1296,7 @@
         <v>4758</v>
       </c>
       <c r="C27" t="n">
-        <v>3806</v>
+        <v>3924</v>
       </c>
       <c r="D27" t="n">
         <v>2</v>
@@ -1198,11 +1308,16 @@
         <v>42650</v>
       </c>
       <c r="G27" t="n">
-        <v>34704</v>
+        <v>37844</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Lv 26: Smooth interpolation (x0.825)</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1329,7 @@
         <v>5160</v>
       </c>
       <c r="C28" t="n">
-        <v>4128</v>
+        <v>4217</v>
       </c>
       <c r="D28" t="n">
         <v>3</v>
@@ -1226,11 +1341,16 @@
         <v>47810</v>
       </c>
       <c r="G28" t="n">
-        <v>38832</v>
+        <v>42061</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Lv 27: Smooth interpolation (x0.817)</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1362,7 @@
         <v>5580</v>
       </c>
       <c r="C29" t="n">
-        <v>4464</v>
+        <v>4522</v>
       </c>
       <c r="D29" t="n">
         <v>3</v>
@@ -1254,11 +1374,16 @@
         <v>53390</v>
       </c>
       <c r="G29" t="n">
-        <v>43296</v>
+        <v>46583</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Lv 28: Smooth interpolation (x0.810)</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1395,7 @@
         <v>6018</v>
       </c>
       <c r="C30" t="n">
-        <v>4814</v>
+        <v>4842</v>
       </c>
       <c r="D30" t="n">
         <v>3</v>
@@ -1282,11 +1407,16 @@
         <v>59408</v>
       </c>
       <c r="G30" t="n">
-        <v>48110</v>
+        <v>51425</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Lv 29: Smooth interpolation (x0.805)</t>
         </is>
       </c>
     </row>
@@ -1310,11 +1440,16 @@
         <v>65882</v>
       </c>
       <c r="G31" t="n">
-        <v>53289</v>
+        <v>56604</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Lv 30: Smooth interpolation (x0.800)</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1461,7 @@
         <v>7295</v>
       </c>
       <c r="C32" t="n">
-        <v>5471</v>
+        <v>5808</v>
       </c>
       <c r="D32" t="n">
         <v>3</v>
@@ -1338,7 +1473,7 @@
         <v>73177</v>
       </c>
       <c r="G32" t="n">
-        <v>58760</v>
+        <v>62412</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -1347,7 +1482,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Lv 31-50: 25% EXP reduction to smooth Advanced Class transition</t>
+          <t>Lv 31: Smooth postgame transition (x0.796)</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1494,7 @@
         <v>7812</v>
       </c>
       <c r="C33" t="n">
-        <v>5859</v>
+        <v>6191</v>
       </c>
       <c r="D33" t="n">
         <v>3</v>
@@ -1371,11 +1506,16 @@
         <v>80989</v>
       </c>
       <c r="G33" t="n">
-        <v>64619</v>
+        <v>68603</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Lv 32: Smooth postgame transition (x0.792)</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1527,7 @@
         <v>8347</v>
       </c>
       <c r="C34" t="n">
-        <v>6260</v>
+        <v>6587</v>
       </c>
       <c r="D34" t="n">
         <v>4</v>
@@ -1399,11 +1539,16 @@
         <v>89336</v>
       </c>
       <c r="G34" t="n">
-        <v>70879</v>
+        <v>75190</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Lv 33: Smooth postgame transition (x0.789)</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1560,7 @@
         <v>8902</v>
       </c>
       <c r="C35" t="n">
-        <v>6676</v>
+        <v>6997</v>
       </c>
       <c r="D35" t="n">
         <v>4</v>
@@ -1427,11 +1572,16 @@
         <v>98238</v>
       </c>
       <c r="G35" t="n">
-        <v>77555</v>
+        <v>82187</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Lv 34: Smooth postgame transition (x0.786)</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1593,7 @@
         <v>9477</v>
       </c>
       <c r="C36" t="n">
-        <v>7108</v>
+        <v>7422</v>
       </c>
       <c r="D36" t="n">
         <v>4</v>
@@ -1455,11 +1605,16 @@
         <v>107715</v>
       </c>
       <c r="G36" t="n">
-        <v>84663</v>
+        <v>89609</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Lv 35: Smooth postgame transition (x0.783)</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1626,7 @@
         <v>10071</v>
       </c>
       <c r="C37" t="n">
-        <v>7553</v>
+        <v>7860</v>
       </c>
       <c r="D37" t="n">
         <v>4</v>
@@ -1483,11 +1638,16 @@
         <v>117786</v>
       </c>
       <c r="G37" t="n">
-        <v>92216</v>
+        <v>97469</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Lv 36: Smooth postgame transition (x0.780)</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1659,7 @@
         <v>10685</v>
       </c>
       <c r="C38" t="n">
-        <v>8014</v>
+        <v>8312</v>
       </c>
       <c r="D38" t="n">
         <v>4</v>
@@ -1511,11 +1671,16 @@
         <v>128471</v>
       </c>
       <c r="G38" t="n">
-        <v>100230</v>
+        <v>105781</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Lv 37: Smooth postgame transition (x0.778)</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1692,7 @@
         <v>11320</v>
       </c>
       <c r="C39" t="n">
-        <v>8490</v>
+        <v>8779</v>
       </c>
       <c r="D39" t="n">
         <v>4</v>
@@ -1539,11 +1704,16 @@
         <v>139791</v>
       </c>
       <c r="G39" t="n">
-        <v>108720</v>
+        <v>114560</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Lv 38: Smooth postgame transition (x0.776)</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1725,7 @@
         <v>11973</v>
       </c>
       <c r="C40" t="n">
-        <v>8980</v>
+        <v>9259</v>
       </c>
       <c r="D40" t="n">
         <v>4</v>
@@ -1567,11 +1737,16 @@
         <v>151764</v>
       </c>
       <c r="G40" t="n">
-        <v>117700</v>
+        <v>123819</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Lv 39: Smooth postgame transition (x0.773)</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1758,7 @@
         <v>12646</v>
       </c>
       <c r="C41" t="n">
-        <v>9484</v>
+        <v>9752</v>
       </c>
       <c r="D41" t="n">
         <v>4</v>
@@ -1595,11 +1770,16 @@
         <v>164410</v>
       </c>
       <c r="G41" t="n">
-        <v>127184</v>
+        <v>133571</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Lv 40: Smooth postgame transition (x0.771)</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1791,7 @@
         <v>13656</v>
       </c>
       <c r="C42" t="n">
-        <v>10242</v>
+        <v>10502</v>
       </c>
       <c r="D42" t="n">
         <v>4</v>
@@ -1623,11 +1803,16 @@
         <v>178066</v>
       </c>
       <c r="G42" t="n">
-        <v>137426</v>
+        <v>144073</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Lv 41: Smooth postgame transition (x0.769)</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1824,7 @@
         <v>14386</v>
       </c>
       <c r="C43" t="n">
-        <v>10790</v>
+        <v>11035</v>
       </c>
       <c r="D43" t="n">
         <v>4</v>
@@ -1651,11 +1836,16 @@
         <v>192452</v>
       </c>
       <c r="G43" t="n">
-        <v>148216</v>
+        <v>155108</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Lv 42: Smooth postgame transition (x0.767)</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1857,7 @@
         <v>15138</v>
       </c>
       <c r="C44" t="n">
-        <v>11354</v>
+        <v>11581</v>
       </c>
       <c r="D44" t="n">
         <v>4</v>
@@ -1679,11 +1869,16 @@
         <v>207590</v>
       </c>
       <c r="G44" t="n">
-        <v>159570</v>
+        <v>166689</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Lv 43: Smooth postgame transition (x0.765)</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1890,7 @@
         <v>15910</v>
       </c>
       <c r="C45" t="n">
-        <v>11932</v>
+        <v>12140</v>
       </c>
       <c r="D45" t="n">
         <v>5</v>
@@ -1707,11 +1902,16 @@
         <v>223500</v>
       </c>
       <c r="G45" t="n">
-        <v>171502</v>
+        <v>178829</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Lv 44: Smooth postgame transition (x0.763)</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1923,7 @@
         <v>16702</v>
       </c>
       <c r="C46" t="n">
-        <v>12526</v>
+        <v>12711</v>
       </c>
       <c r="D46" t="n">
         <v>5</v>
@@ -1735,11 +1935,16 @@
         <v>240202</v>
       </c>
       <c r="G46" t="n">
-        <v>184028</v>
+        <v>191540</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Lv 45: Smooth postgame transition (x0.761)</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1956,7 @@
         <v>17514</v>
       </c>
       <c r="C47" t="n">
-        <v>13136</v>
+        <v>13293</v>
       </c>
       <c r="D47" t="n">
         <v>5</v>
@@ -1763,11 +1968,16 @@
         <v>257716</v>
       </c>
       <c r="G47" t="n">
-        <v>197164</v>
+        <v>204833</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Lv 46: Smooth postgame transition (x0.759)</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1989,7 @@
         <v>18349</v>
       </c>
       <c r="C48" t="n">
-        <v>13762</v>
+        <v>13889</v>
       </c>
       <c r="D48" t="n">
         <v>5</v>
@@ -1791,11 +2001,16 @@
         <v>276065</v>
       </c>
       <c r="G48" t="n">
-        <v>210926</v>
+        <v>218722</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Lv 47: Smooth postgame transition (x0.757)</t>
         </is>
       </c>
     </row>
@@ -1807,7 +2022,7 @@
         <v>19203</v>
       </c>
       <c r="C49" t="n">
-        <v>14402</v>
+        <v>14493</v>
       </c>
       <c r="D49" t="n">
         <v>5</v>
@@ -1819,11 +2034,16 @@
         <v>295268</v>
       </c>
       <c r="G49" t="n">
-        <v>225328</v>
+        <v>233215</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Lv 48: Smooth postgame transition (x0.755)</t>
         </is>
       </c>
     </row>
@@ -1835,7 +2055,7 @@
         <v>20079</v>
       </c>
       <c r="C50" t="n">
-        <v>15059</v>
+        <v>15108</v>
       </c>
       <c r="D50" t="n">
         <v>6</v>
@@ -1847,11 +2067,16 @@
         <v>315347</v>
       </c>
       <c r="G50" t="n">
-        <v>240387</v>
+        <v>248323</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Lv 49: Smooth postgame transition (x0.752)</t>
         </is>
       </c>
     </row>
@@ -1875,11 +2100,16 @@
         <v>336323</v>
       </c>
       <c r="G51" t="n">
-        <v>256119</v>
+        <v>264055</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Lv 50: Smooth postgame transition (x0.750)</t>
         </is>
       </c>
     </row>
@@ -1891,7 +2121,7 @@
         <v>22403</v>
       </c>
       <c r="C52" t="n">
-        <v>16802</v>
+        <v>16747</v>
       </c>
       <c r="D52" t="n">
         <v>6</v>
@@ -1903,7 +2133,7 @@
         <v>358726</v>
       </c>
       <c r="G52" t="n">
-        <v>272921</v>
+        <v>280802</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -1912,7 +2142,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Lv 51-70: 25% EXP reduction</t>
+          <t>Lv 51: Smooth postgame transition (x0.748)</t>
         </is>
       </c>
     </row>
@@ -1924,7 +2154,7 @@
         <v>23365</v>
       </c>
       <c r="C53" t="n">
-        <v>17524</v>
+        <v>17409</v>
       </c>
       <c r="D53" t="n">
         <v>6</v>
@@ -1936,11 +2166,16 @@
         <v>382091</v>
       </c>
       <c r="G53" t="n">
-        <v>290445</v>
+        <v>298211</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Lv 52: Smooth postgame transition (x0.745)</t>
         </is>
       </c>
     </row>
@@ -1952,7 +2187,7 @@
         <v>24348</v>
       </c>
       <c r="C54" t="n">
-        <v>18261</v>
+        <v>18082</v>
       </c>
       <c r="D54" t="n">
         <v>6</v>
@@ -1964,11 +2199,16 @@
         <v>406439</v>
       </c>
       <c r="G54" t="n">
-        <v>308706</v>
+        <v>316293</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Lv 53: Smooth postgame transition (x0.743)</t>
         </is>
       </c>
     </row>
@@ -1980,7 +2220,7 @@
         <v>25352</v>
       </c>
       <c r="C55" t="n">
-        <v>19014</v>
+        <v>18767</v>
       </c>
       <c r="D55" t="n">
         <v>7</v>
@@ -1992,11 +2232,16 @@
         <v>431791</v>
       </c>
       <c r="G55" t="n">
-        <v>327720</v>
+        <v>335060</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Lv 54: Smooth postgame transition (x0.740)</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2253,7 @@
         <v>26379</v>
       </c>
       <c r="C56" t="n">
-        <v>19784</v>
+        <v>19464</v>
       </c>
       <c r="D56" t="n">
         <v>7</v>
@@ -2020,11 +2265,16 @@
         <v>458170</v>
       </c>
       <c r="G56" t="n">
-        <v>347504</v>
+        <v>354524</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Lv 55: Smooth postgame transition (x0.738)</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2286,7 @@
         <v>27427</v>
       </c>
       <c r="C57" t="n">
-        <v>20570</v>
+        <v>20172</v>
       </c>
       <c r="D57" t="n">
         <v>7</v>
@@ -2048,11 +2298,16 @@
         <v>485597</v>
       </c>
       <c r="G57" t="n">
-        <v>368074</v>
+        <v>374696</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Lv 56: Smooth postgame transition (x0.735)</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2319,7 @@
         <v>28497</v>
       </c>
       <c r="C58" t="n">
-        <v>21373</v>
+        <v>20891</v>
       </c>
       <c r="D58" t="n">
         <v>7</v>
@@ -2076,11 +2331,16 @@
         <v>514094</v>
       </c>
       <c r="G58" t="n">
-        <v>389447</v>
+        <v>395587</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Lv 57: Smooth postgame transition (x0.733)</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2352,7 @@
         <v>29590</v>
       </c>
       <c r="C59" t="n">
-        <v>22192</v>
+        <v>21622</v>
       </c>
       <c r="D59" t="n">
         <v>7</v>
@@ -2104,11 +2364,16 @@
         <v>543684</v>
       </c>
       <c r="G59" t="n">
-        <v>411639</v>
+        <v>417209</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Lv 58: Smooth postgame transition (x0.731)</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2385,7 @@
         <v>30704</v>
       </c>
       <c r="C60" t="n">
-        <v>23028</v>
+        <v>22363</v>
       </c>
       <c r="D60" t="n">
         <v>7</v>
@@ -2132,11 +2397,16 @@
         <v>574388</v>
       </c>
       <c r="G60" t="n">
-        <v>434667</v>
+        <v>439572</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Lv 59: Smooth postgame transition (x0.728)</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2418,7 @@
         <v>31841</v>
       </c>
       <c r="C61" t="n">
-        <v>23881</v>
+        <v>23115</v>
       </c>
       <c r="D61" t="n">
         <v>8</v>
@@ -2160,11 +2430,16 @@
         <v>606229</v>
       </c>
       <c r="G61" t="n">
-        <v>458548</v>
+        <v>462687</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Lv 60: Smooth postgame transition (x0.726)</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2451,7 @@
         <v>33001</v>
       </c>
       <c r="C62" t="n">
-        <v>21451</v>
+        <v>23877</v>
       </c>
       <c r="D62" t="n">
         <v>8</v>
@@ -2188,7 +2463,7 @@
         <v>639230</v>
       </c>
       <c r="G62" t="n">
-        <v>479999</v>
+        <v>486564</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -2197,7 +2472,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 61: Smooth postgame transition (x0.724)</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2484,7 @@
         <v>34182</v>
       </c>
       <c r="C63" t="n">
-        <v>22218</v>
+        <v>24648</v>
       </c>
       <c r="D63" t="n">
         <v>8</v>
@@ -2221,7 +2496,7 @@
         <v>673412</v>
       </c>
       <c r="G63" t="n">
-        <v>502217</v>
+        <v>511212</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -2230,7 +2505,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 62: Smooth postgame transition (x0.721)</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2517,7 @@
         <v>35385</v>
       </c>
       <c r="C64" t="n">
-        <v>23000</v>
+        <v>25428</v>
       </c>
       <c r="D64" t="n">
         <v>8</v>
@@ -2254,7 +2529,7 @@
         <v>708797</v>
       </c>
       <c r="G64" t="n">
-        <v>525217</v>
+        <v>536640</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -2263,7 +2538,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 63: Smooth postgame transition (x0.719)</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2550,7 @@
         <v>36612</v>
       </c>
       <c r="C65" t="n">
-        <v>23798</v>
+        <v>26218</v>
       </c>
       <c r="D65" t="n">
         <v>8</v>
@@ -2287,7 +2562,7 @@
         <v>745409</v>
       </c>
       <c r="G65" t="n">
-        <v>549015</v>
+        <v>562858</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -2296,7 +2571,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 64: Smooth postgame transition (x0.716)</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2583,7 @@
         <v>37860</v>
       </c>
       <c r="C66" t="n">
-        <v>24609</v>
+        <v>27015</v>
       </c>
       <c r="D66" t="n">
         <v>9</v>
@@ -2320,7 +2595,7 @@
         <v>783269</v>
       </c>
       <c r="G66" t="n">
-        <v>573624</v>
+        <v>589873</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -2329,7 +2604,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 65: Smooth postgame transition (x0.714)</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2616,7 @@
         <v>39132</v>
       </c>
       <c r="C67" t="n">
-        <v>25436</v>
+        <v>27821</v>
       </c>
       <c r="D67" t="n">
         <v>9</v>
@@ -2353,7 +2628,7 @@
         <v>822401</v>
       </c>
       <c r="G67" t="n">
-        <v>599060</v>
+        <v>617694</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -2362,7 +2637,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 66: Smooth postgame transition (x0.711)</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2649,7 @@
         <v>40426</v>
       </c>
       <c r="C68" t="n">
-        <v>26277</v>
+        <v>28634</v>
       </c>
       <c r="D68" t="n">
         <v>9</v>
@@ -2386,7 +2661,7 @@
         <v>862827</v>
       </c>
       <c r="G68" t="n">
-        <v>625337</v>
+        <v>646328</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -2395,7 +2670,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 67: Smooth postgame transition (x0.708)</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2682,7 @@
         <v>41742</v>
       </c>
       <c r="C69" t="n">
-        <v>27132</v>
+        <v>29454</v>
       </c>
       <c r="D69" t="n">
         <v>9</v>
@@ -2419,7 +2694,7 @@
         <v>904569</v>
       </c>
       <c r="G69" t="n">
-        <v>652469</v>
+        <v>675782</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -2428,7 +2703,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 68: Smooth postgame transition (x0.706)</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2715,7 @@
         <v>43081</v>
       </c>
       <c r="C70" t="n">
-        <v>28003</v>
+        <v>30279</v>
       </c>
       <c r="D70" t="n">
         <v>10</v>
@@ -2452,7 +2727,7 @@
         <v>947650</v>
       </c>
       <c r="G70" t="n">
-        <v>680472</v>
+        <v>706061</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -2461,7 +2736,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 69: Smooth postgame transition (x0.703)</t>
         </is>
       </c>
     </row>
@@ -2473,7 +2748,7 @@
         <v>44443</v>
       </c>
       <c r="C71" t="n">
-        <v>28888</v>
+        <v>31110</v>
       </c>
       <c r="D71" t="n">
         <v>10</v>
@@ -2485,7 +2760,7 @@
         <v>992093</v>
       </c>
       <c r="G71" t="n">
-        <v>709360</v>
+        <v>737171</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -2494,7 +2769,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Lv 61-70: -35% postgame transition</t>
+          <t>Lv 70: Smooth postgame transition (x0.700)</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2781,7 @@
         <v>45828</v>
       </c>
       <c r="C72" t="n">
-        <v>34371</v>
+        <v>31945</v>
       </c>
       <c r="D72" t="n">
         <v>10</v>
@@ -2518,7 +2793,7 @@
         <v>1037921</v>
       </c>
       <c r="G72" t="n">
-        <v>743731</v>
+        <v>769116</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -2527,7 +2802,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 71: Calibrated ~1h endgame climb (x0.697)</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2814,7 @@
         <v>47236</v>
       </c>
       <c r="C73" t="n">
-        <v>35427</v>
+        <v>32784</v>
       </c>
       <c r="D73" t="n">
         <v>10</v>
@@ -2551,7 +2826,7 @@
         <v>1085157</v>
       </c>
       <c r="G73" t="n">
-        <v>779158</v>
+        <v>801900</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -2560,7 +2835,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 72: Calibrated ~1h endgame climb (x0.694)</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2847,7 @@
         <v>48666</v>
       </c>
       <c r="C74" t="n">
-        <v>36500</v>
+        <v>33625</v>
       </c>
       <c r="D74" t="n">
         <v>10</v>
@@ -2584,7 +2859,7 @@
         <v>1133823</v>
       </c>
       <c r="G74" t="n">
-        <v>815658</v>
+        <v>835525</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -2593,7 +2868,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 73: Calibrated ~1h endgame climb (x0.691)</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2880,7 @@
         <v>50119</v>
       </c>
       <c r="C75" t="n">
-        <v>37589</v>
+        <v>34469</v>
       </c>
       <c r="D75" t="n">
         <v>11</v>
@@ -2617,7 +2892,7 @@
         <v>1183942</v>
       </c>
       <c r="G75" t="n">
-        <v>853247</v>
+        <v>869994</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -2626,7 +2901,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 74: Calibrated ~1h endgame climb (x0.688)</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2913,7 @@
         <v>51595</v>
       </c>
       <c r="C76" t="n">
-        <v>38696</v>
+        <v>35316</v>
       </c>
       <c r="D76" t="n">
         <v>11</v>
@@ -2650,7 +2925,7 @@
         <v>1235537</v>
       </c>
       <c r="G76" t="n">
-        <v>891943</v>
+        <v>905310</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -2659,7 +2934,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 75: Calibrated ~1h endgame climb (x0.684)</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2946,7 @@
         <v>53094</v>
       </c>
       <c r="C77" t="n">
-        <v>39820</v>
+        <v>36165</v>
       </c>
       <c r="D77" t="n">
         <v>11</v>
@@ -2683,7 +2958,7 @@
         <v>1288631</v>
       </c>
       <c r="G77" t="n">
-        <v>931763</v>
+        <v>941475</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -2692,7 +2967,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 76: Calibrated ~1h endgame climb (x0.681)</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2979,7 @@
         <v>54617</v>
       </c>
       <c r="C78" t="n">
-        <v>40963</v>
+        <v>37018</v>
       </c>
       <c r="D78" t="n">
         <v>11</v>
@@ -2716,7 +2991,7 @@
         <v>1343248</v>
       </c>
       <c r="G78" t="n">
-        <v>972726</v>
+        <v>978493</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -2725,7 +3000,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 77: Calibrated ~1h endgame climb (x0.678)</t>
         </is>
       </c>
     </row>
@@ -2737,7 +3012,7 @@
         <v>56162</v>
       </c>
       <c r="C79" t="n">
-        <v>42122</v>
+        <v>37873</v>
       </c>
       <c r="D79" t="n">
         <v>12</v>
@@ -2749,7 +3024,7 @@
         <v>1399410</v>
       </c>
       <c r="G79" t="n">
-        <v>1014848</v>
+        <v>1016366</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -2758,7 +3033,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 78: Calibrated ~1h endgame climb (x0.674)</t>
         </is>
       </c>
     </row>
@@ -2770,7 +3045,7 @@
         <v>57731</v>
       </c>
       <c r="C80" t="n">
-        <v>43298</v>
+        <v>38732</v>
       </c>
       <c r="D80" t="n">
         <v>12</v>
@@ -2782,7 +3057,7 @@
         <v>1457141</v>
       </c>
       <c r="G80" t="n">
-        <v>1058146</v>
+        <v>1055098</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -2791,7 +3066,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 79: Calibrated ~1h endgame climb (x0.671)</t>
         </is>
       </c>
     </row>
@@ -2803,7 +3078,7 @@
         <v>59323</v>
       </c>
       <c r="C81" t="n">
-        <v>44492</v>
+        <v>39594</v>
       </c>
       <c r="D81" t="n">
         <v>12</v>
@@ -2815,7 +3090,7 @@
         <v>1516464</v>
       </c>
       <c r="G81" t="n">
-        <v>1102638</v>
+        <v>1094692</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -2824,7 +3099,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 80: Calibrated ~1h endgame climb (x0.667)</t>
         </is>
       </c>
     </row>
@@ -2836,7 +3111,7 @@
         <v>62322</v>
       </c>
       <c r="C82" t="n">
-        <v>46742</v>
+        <v>41378</v>
       </c>
       <c r="D82" t="n">
         <v>12</v>
@@ -2848,7 +3123,7 @@
         <v>1578786</v>
       </c>
       <c r="G82" t="n">
-        <v>1149380</v>
+        <v>1136070</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -2857,7 +3132,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 81: Calibrated ~1h endgame climb (x0.664)</t>
         </is>
       </c>
     </row>
@@ -2869,7 +3144,7 @@
         <v>63997</v>
       </c>
       <c r="C83" t="n">
-        <v>47998</v>
+        <v>42266</v>
       </c>
       <c r="D83" t="n">
         <v>13</v>
@@ -2881,7 +3156,7 @@
         <v>1642783</v>
       </c>
       <c r="G83" t="n">
-        <v>1197378</v>
+        <v>1178336</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -2890,7 +3165,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 82: Calibrated ~1h endgame climb (x0.660)</t>
         </is>
       </c>
     </row>
@@ -2902,7 +3177,7 @@
         <v>65697</v>
       </c>
       <c r="C84" t="n">
-        <v>49273</v>
+        <v>43159</v>
       </c>
       <c r="D84" t="n">
         <v>13</v>
@@ -2914,7 +3189,7 @@
         <v>1708480</v>
       </c>
       <c r="G84" t="n">
-        <v>1246651</v>
+        <v>1221495</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -2923,7 +3198,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 83: Calibrated ~1h endgame climb (x0.657)</t>
         </is>
       </c>
     </row>
@@ -2935,7 +3210,7 @@
         <v>67421</v>
       </c>
       <c r="C85" t="n">
-        <v>50566</v>
+        <v>44057</v>
       </c>
       <c r="D85" t="n">
         <v>13</v>
@@ -2947,7 +3222,7 @@
         <v>1775901</v>
       </c>
       <c r="G85" t="n">
-        <v>1297217</v>
+        <v>1265552</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -2956,7 +3231,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 84: Calibrated ~1h endgame climb (x0.653)</t>
         </is>
       </c>
     </row>
@@ -2968,7 +3243,7 @@
         <v>69783</v>
       </c>
       <c r="C86" t="n">
-        <v>52337</v>
+        <v>45359</v>
       </c>
       <c r="D86" t="n">
         <v>13</v>
@@ -2980,7 +3255,7 @@
         <v>1845684</v>
       </c>
       <c r="G86" t="n">
-        <v>1349554</v>
+        <v>1310911</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -2989,7 +3264,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Lv 71-85: -25% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 85: Calibrated ~1h endgame climb (x0.650)</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3276,7 @@
         <v>71569</v>
       </c>
       <c r="C87" t="n">
-        <v>42941</v>
+        <v>46272</v>
       </c>
       <c r="D87" t="n">
         <v>14</v>
@@ -3013,7 +3288,7 @@
         <v>1917253</v>
       </c>
       <c r="G87" t="n">
-        <v>1392495</v>
+        <v>1357183</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -3022,7 +3297,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 86: Calibrated ~1h endgame climb (x0.647)</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3309,7 @@
         <v>73381</v>
       </c>
       <c r="C88" t="n">
-        <v>44029</v>
+        <v>47189</v>
       </c>
       <c r="D88" t="n">
         <v>14</v>
@@ -3046,7 +3321,7 @@
         <v>1990634</v>
       </c>
       <c r="G88" t="n">
-        <v>1436524</v>
+        <v>1404372</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -3055,7 +3330,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 87: Calibrated ~1h endgame climb (x0.643)</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3342,7 @@
         <v>75216</v>
       </c>
       <c r="C89" t="n">
-        <v>45130</v>
+        <v>48106</v>
       </c>
       <c r="D89" t="n">
         <v>14</v>
@@ -3079,7 +3354,7 @@
         <v>2065850</v>
       </c>
       <c r="G89" t="n">
-        <v>1481654</v>
+        <v>1452478</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -3088,7 +3363,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 88: Calibrated ~1h endgame climb (x0.640)</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3375,7 @@
         <v>77076</v>
       </c>
       <c r="C90" t="n">
-        <v>46246</v>
+        <v>49025</v>
       </c>
       <c r="D90" t="n">
         <v>14</v>
@@ -3112,7 +3387,7 @@
         <v>2142926</v>
       </c>
       <c r="G90" t="n">
-        <v>1527900</v>
+        <v>1501503</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -3121,7 +3396,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 89: Calibrated ~1h endgame climb (x0.636)</t>
         </is>
       </c>
     </row>
@@ -3133,7 +3408,7 @@
         <v>78960</v>
       </c>
       <c r="C91" t="n">
-        <v>47376</v>
+        <v>49944</v>
       </c>
       <c r="D91" t="n">
         <v>15</v>
@@ -3145,7 +3420,7 @@
         <v>2221886</v>
       </c>
       <c r="G91" t="n">
-        <v>1575276</v>
+        <v>1551447</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -3154,7 +3429,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 90: Calibrated ~1h endgame climb (x0.633)</t>
         </is>
       </c>
     </row>
@@ -3166,7 +3441,7 @@
         <v>81938</v>
       </c>
       <c r="C92" t="n">
-        <v>49163</v>
+        <v>51537</v>
       </c>
       <c r="D92" t="n">
         <v>15</v>
@@ -3178,7 +3453,7 @@
         <v>2303824</v>
       </c>
       <c r="G92" t="n">
-        <v>1624439</v>
+        <v>1602984</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -3187,7 +3462,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 91: Calibrated ~1h endgame climb (x0.629)</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3474,7 @@
         <v>83897</v>
       </c>
       <c r="C93" t="n">
-        <v>50338</v>
+        <v>52470</v>
       </c>
       <c r="D93" t="n">
         <v>15</v>
@@ -3211,7 +3486,7 @@
         <v>2387721</v>
       </c>
       <c r="G93" t="n">
-        <v>1674777</v>
+        <v>1655454</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -3220,7 +3495,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 92: Calibrated ~1h endgame climb (x0.625)</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3507,7 @@
         <v>85880</v>
       </c>
       <c r="C94" t="n">
-        <v>51528</v>
+        <v>53403</v>
       </c>
       <c r="D94" t="n">
         <v>15</v>
@@ -3244,7 +3519,7 @@
         <v>2473601</v>
       </c>
       <c r="G94" t="n">
-        <v>1726305</v>
+        <v>1708857</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -3253,7 +3528,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 93: Calibrated ~1h endgame climb (x0.622)</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3540,7 @@
         <v>87888</v>
       </c>
       <c r="C95" t="n">
-        <v>52733</v>
+        <v>54335</v>
       </c>
       <c r="D95" t="n">
         <v>16</v>
@@ -3277,7 +3552,7 @@
         <v>2561489</v>
       </c>
       <c r="G95" t="n">
-        <v>1779038</v>
+        <v>1763192</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -3286,7 +3561,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 94: Calibrated ~1h endgame climb (x0.618)</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3573,7 @@
         <v>91876</v>
       </c>
       <c r="C96" t="n">
-        <v>55126</v>
+        <v>56469</v>
       </c>
       <c r="D96" t="n">
         <v>16</v>
@@ -3310,7 +3585,7 @@
         <v>2653365</v>
       </c>
       <c r="G96" t="n">
-        <v>1834164</v>
+        <v>1819661</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -3319,7 +3594,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 95: Calibrated ~1h endgame climb (x0.615)</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3606,7 @@
         <v>93980</v>
       </c>
       <c r="C97" t="n">
-        <v>56388</v>
+        <v>57421</v>
       </c>
       <c r="D97" t="n">
         <v>16</v>
@@ -3343,7 +3618,7 @@
         <v>2747345</v>
       </c>
       <c r="G97" t="n">
-        <v>1890552</v>
+        <v>1877082</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -3352,7 +3627,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 96: Calibrated ~1h endgame climb (x0.611)</t>
         </is>
       </c>
     </row>
@@ -3364,7 +3639,7 @@
         <v>96109</v>
       </c>
       <c r="C98" t="n">
-        <v>57665</v>
+        <v>58371</v>
       </c>
       <c r="D98" t="n">
         <v>17</v>
@@ -3376,7 +3651,7 @@
         <v>2843454</v>
       </c>
       <c r="G98" t="n">
-        <v>1948217</v>
+        <v>1935453</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -3385,7 +3660,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 97: Calibrated ~1h endgame climb (x0.607)</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3672,7 @@
         <v>98262</v>
       </c>
       <c r="C99" t="n">
-        <v>58957</v>
+        <v>59319</v>
       </c>
       <c r="D99" t="n">
         <v>17</v>
@@ -3409,7 +3684,7 @@
         <v>2941716</v>
       </c>
       <c r="G99" t="n">
-        <v>2007174</v>
+        <v>1994772</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -3418,7 +3693,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 98: Calibrated ~1h endgame climb (x0.604)</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3717,7 @@
         <v>3042158</v>
       </c>
       <c r="G100" t="n">
-        <v>2067439</v>
+        <v>2055037</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -3451,7 +3726,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Lv 86-99: -40% EXP tuned for ~1h climb to Lv 99</t>
+          <t>Lv 99: Calibrated ~1h endgame climb (x0.600)</t>
         </is>
       </c>
     </row>

</xml_diff>